<commit_message>
working on last test to work
</commit_message>
<xml_diff>
--- a/test/configs/data/test/3n_3c_1gext_1h_1bext_2l.xlsx
+++ b/test/configs/data/test/3n_3c_1gext_1h_1bext_2l.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="154">
   <si>
     <t>name</t>
   </si>
@@ -485,6 +485,9 @@
   </si>
   <si>
     <t>IT0 0 H2 Fuel Cell</t>
+  </si>
+  <si>
+    <t>line 0-1</t>
   </si>
 </sst>
 </file>
@@ -1296,7 +1299,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AJ2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="4" width="8.88671875" style="5" bestFit="1" customWidth="1"/>
@@ -1412,6 +1415,38 @@
       </c>
       <c r="AJ1" t="s">
         <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E2" s="5">
+        <v>5</v>
+      </c>
+      <c r="F2" s="5">
+        <v>0.1</v>
+      </c>
+      <c r="I2">
+        <v>100</v>
+      </c>
+      <c r="K2" t="s">
+        <v>30</v>
+      </c>
+      <c r="L2">
+        <v>100</v>
+      </c>
+      <c r="M2">
+        <v>10000</v>
+      </c>
+      <c r="P2">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>